<commit_message>
Update PhoneSpot Codex system 2026-06-24 13:55
</commit_message>
<xml_diff>
--- a/_preview_dashboard.xlsx
+++ b/_preview_dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합대시보드_미리보기" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'통합대시보드_미리보기'!$A$1:$M$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'통합대시보드_미리보기'!$A$1:$N$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -569,12 +569,13 @@
     <col width="11.4" customWidth="1" min="5" max="5"/>
     <col width="11.4" customWidth="1" min="6" max="6"/>
     <col width="11.4" customWidth="1" min="7" max="7"/>
-    <col width="15.7" customWidth="1" min="8" max="8"/>
-    <col width="15.4" customWidth="1" min="9" max="9"/>
+    <col width="3.6" customWidth="1" min="8" max="8"/>
+    <col width="15.7" customWidth="1" min="9" max="9"/>
     <col width="15.4" customWidth="1" min="10" max="10"/>
     <col width="15.4" customWidth="1" min="11" max="11"/>
     <col width="15.4" customWidth="1" min="12" max="12"/>
     <col width="15.4" customWidth="1" min="13" max="13"/>
+    <col width="15.4" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -655,7 +656,7 @@
           <t>기간별 핵심</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr">
         <is>
           <t>SNS 채널 운영</t>
         </is>
@@ -692,32 +693,32 @@
           <t>순이익</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>채널</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>포스트수</t>
         </is>
       </c>
-      <c r="J5" s="11" t="inlineStr">
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>총조회수</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="L5" s="11" t="inlineStr">
         <is>
           <t>평균</t>
         </is>
       </c>
-      <c r="L5" s="11" t="inlineStr">
+      <c r="M5" s="11" t="inlineStr">
         <is>
           <t>팔로워</t>
         </is>
       </c>
-      <c r="M5" s="11" t="inlineStr"/>
+      <c r="N5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -742,21 +743,21 @@
       <c r="F6" s="13" t="n">
         <v>13616</v>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="I6" s="12" t="inlineStr">
         <is>
           <t>유튜브</t>
         </is>
       </c>
-      <c r="I6" s="14" t="n">
+      <c r="J6" s="14" t="n">
         <v>41</v>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="K6" s="14" t="n">
         <v>17177</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="14" t="n">
         <v>419</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="14" t="n">
         <v>12</v>
       </c>
     </row>
@@ -781,21 +782,21 @@
       <c r="F7" s="16" t="n">
         <v>-207913</v>
       </c>
-      <c r="H7" s="15" t="inlineStr">
+      <c r="I7" s="15" t="inlineStr">
         <is>
           <t>인스타</t>
         </is>
       </c>
-      <c r="I7" s="17" t="n">
+      <c r="J7" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="J7" s="17" t="n">
+      <c r="K7" s="17" t="n">
         <v>1395</v>
       </c>
-      <c r="K7" s="17" t="n">
+      <c r="L7" s="17" t="n">
         <v>100</v>
       </c>
-      <c r="L7" s="17" t="n">
+      <c r="M7" s="17" t="n">
         <v>64</v>
       </c>
     </row>
@@ -820,40 +821,40 @@
       <c r="F8" s="13" t="n">
         <v>-1560347</v>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>스레드</t>
         </is>
       </c>
-      <c r="I8" s="14" t="n">
+      <c r="J8" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="J8" s="14" t="n">
+      <c r="K8" s="14" t="n">
         <v>364</v>
       </c>
-      <c r="K8" s="14" t="n">
+      <c r="L8" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="L8" s="14" t="n">
+      <c r="M8" s="14" t="n">
         <v>137</v>
       </c>
     </row>
     <row r="9">
-      <c r="H9" s="15" t="inlineStr">
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>틱톡</t>
         </is>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="J9" s="17" t="n">
         <v>31</v>
       </c>
-      <c r="J9" s="17" t="n">
+      <c r="K9" s="17" t="n">
         <v>2286</v>
       </c>
-      <c r="K9" s="17" t="n">
+      <c r="L9" s="17" t="n">
         <v>74</v>
       </c>
-      <c r="L9" s="17" t="n">
+      <c r="M9" s="17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -863,7 +864,7 @@
           <t>채널별 효율</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>실비용 대조 (이번달 카드결제 vs API 광고비)</t>
         </is>
@@ -905,28 +906,28 @@
           <t>앱문의</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="I11" s="11" t="inlineStr">
         <is>
           <t>채널</t>
         </is>
       </c>
-      <c r="I11" s="11" t="inlineStr">
+      <c r="J11" s="11" t="inlineStr">
         <is>
           <t>카드결제</t>
         </is>
       </c>
-      <c r="J11" s="11" t="inlineStr">
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>API광고비</t>
         </is>
       </c>
-      <c r="K11" s="11" t="inlineStr">
+      <c r="L11" s="11" t="inlineStr">
         <is>
           <t>차이</t>
         </is>
       </c>
-      <c r="L11" s="11" t="inlineStr"/>
       <c r="M11" s="11" t="inlineStr"/>
+      <c r="N11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -954,18 +955,18 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr">
         <is>
           <t>메타</t>
         </is>
       </c>
-      <c r="I12" s="13" t="n">
+      <c r="J12" s="13" t="n">
         <v>1450000</v>
       </c>
-      <c r="J12" s="13" t="n">
+      <c r="K12" s="13" t="n">
         <v>1419445</v>
       </c>
-      <c r="K12" s="13" t="n">
+      <c r="L12" s="13" t="n">
         <v>30555</v>
       </c>
     </row>
@@ -995,18 +996,18 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H13" s="15" t="inlineStr">
+      <c r="I13" s="15" t="inlineStr">
         <is>
           <t>네이버</t>
         </is>
       </c>
-      <c r="I13" s="16" t="n">
+      <c r="J13" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="16" t="n">
+      <c r="K13" s="16" t="n">
         <v>6759</v>
       </c>
-      <c r="K13" s="16" t="n">
+      <c r="L13" s="16" t="n">
         <v>-6759</v>
       </c>
     </row>
@@ -1036,18 +1037,18 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="I14" s="12" t="inlineStr">
         <is>
           <t>구글</t>
         </is>
       </c>
-      <c r="I14" s="13" t="n">
+      <c r="J14" s="13" t="n">
         <v>90000</v>
       </c>
-      <c r="J14" s="13" t="n">
+      <c r="K14" s="13" t="n">
         <v>73281</v>
       </c>
-      <c r="K14" s="13" t="n">
+      <c r="L14" s="13" t="n">
         <v>16719</v>
       </c>
     </row>
@@ -1079,13 +1080,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H15" s="15" t="inlineStr">
+      <c r="I15" s="15" t="inlineStr">
         <is>
           <t>카카오</t>
         </is>
-      </c>
-      <c r="I15" s="16" t="n">
-        <v>0</v>
       </c>
       <c r="J15" s="16" t="n">
         <v>0</v>
@@ -1093,6 +1091,9 @@
       <c r="K15" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="L15" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -1118,193 +1119,193 @@
       <c r="G16" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="I16" s="12" t="inlineStr">
         <is>
           <t>당근</t>
         </is>
       </c>
-      <c r="I16" s="13" t="n">
+      <c r="J16" s="13" t="n">
         <v>740000</v>
       </c>
-      <c r="J16" s="13" t="n">
+      <c r="K16" s="13" t="n">
         <v>475328</v>
       </c>
-      <c r="K16" s="13" t="n">
+      <c r="L16" s="13" t="n">
         <v>264672</v>
       </c>
     </row>
     <row r="17">
-      <c r="H17" s="15" t="inlineStr">
+      <c r="I17" s="15" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="I17" s="16" t="n">
+      <c r="J17" s="16" t="n">
         <v>2280000</v>
       </c>
-      <c r="J17" s="16" t="n">
+      <c r="K17" s="16" t="n">
         <v>1974813</v>
       </c>
-      <c r="K17" s="16" t="n">
+      <c r="L17" s="16" t="n">
         <v>305187</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>· 차이(+) = 카드결제가 API 집계보다 큼 (수수료·부가세·미집계분 등)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>리틀리 유입</t>
         </is>
       </c>
-      <c r="H18" s="18" t="inlineStr">
-        <is>
-          <t>· 차이(+) = 카드결제가 API 집계보다 큼 (수수료·부가세·미집계분 등)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>카톡 현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>기간</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>방문자수</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>클릭수</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>CTR</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>최신 유입경로비율</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr"/>
-      <c r="G19" s="11" t="inlineStr"/>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>카톡 현황</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr"/>
+      <c r="G20" s="11" t="inlineStr"/>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>기간</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>광고비</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>카톡클릭</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="inlineStr">
+        <is>
+          <t>카톡당비용</t>
+        </is>
+      </c>
+      <c r="M20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>어제</t>
         </is>
       </c>
-      <c r="B20" s="14" t="n">
+      <c r="B21" s="14" t="n">
         <v>802</v>
       </c>
-      <c r="C20" s="14" t="n">
+      <c r="C21" s="14" t="n">
         <v>288</v>
       </c>
-      <c r="D20" s="19" t="n">
+      <c r="D21" s="19" t="n">
         <v>0.359</v>
       </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>기간</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>광고비</t>
-        </is>
-      </c>
-      <c r="J20" s="11" t="inlineStr">
-        <is>
-          <t>카톡클릭</t>
-        </is>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
-        <is>
-          <t>카톡당비용</t>
-        </is>
-      </c>
-      <c r="L20" s="11" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>어제</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="n">
+        <v>66384</v>
+      </c>
+      <c r="K21" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="L21" s="13" t="n">
+        <v>1660</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>최근 7일</t>
         </is>
       </c>
-      <c r="B21" s="17" t="n">
+      <c r="B22" s="17" t="n">
         <v>4028</v>
       </c>
-      <c r="C21" s="17" t="n">
+      <c r="C22" s="17" t="n">
         <v>1310</v>
       </c>
-      <c r="D21" s="20" t="n">
+      <c r="D22" s="20" t="n">
         <v>0.325</v>
       </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>어제</t>
-        </is>
-      </c>
-      <c r="I21" s="13" t="n">
-        <v>66384</v>
-      </c>
-      <c r="J21" s="14" t="n">
-        <v>40</v>
-      </c>
-      <c r="K21" s="13" t="n">
-        <v>1660</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="I22" s="15" t="inlineStr">
+        <is>
+          <t>최근 7일</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="n">
+        <v>447913</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>292</v>
+      </c>
+      <c r="L22" s="16" t="n">
+        <v>1534</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>최근 30일</t>
         </is>
       </c>
-      <c r="B22" s="14" t="n">
+      <c r="B23" s="14" t="n">
         <v>26297</v>
       </c>
-      <c r="C22" s="14" t="n">
+      <c r="C23" s="14" t="n">
         <v>5973</v>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D23" s="19" t="n">
         <v>0.227</v>
       </c>
-      <c r="H22" s="15" t="inlineStr">
-        <is>
-          <t>최근 7일</t>
-        </is>
-      </c>
-      <c r="I22" s="16" t="n">
-        <v>447913</v>
-      </c>
-      <c r="J22" s="17" t="n">
-        <v>292</v>
-      </c>
-      <c r="K22" s="16" t="n">
-        <v>1534</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="H23" s="12" t="inlineStr">
+      <c r="I23" s="12" t="inlineStr">
         <is>
           <t>최근 30일</t>
         </is>
       </c>
-      <c r="I23" s="13" t="n">
+      <c r="J23" s="13" t="n">
         <v>2680347</v>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="K23" s="14" t="n">
         <v>1252</v>
       </c>
-      <c r="K23" s="13" t="n">
+      <c r="L23" s="13" t="n">
         <v>2141</v>
       </c>
     </row>
@@ -1483,20 +1484,20 @@
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="C1:D1"/>
-    <mergeCell ref="H19:M19"/>
     <mergeCell ref="E1:F1"/>
+    <mergeCell ref="I4:N4"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="I19:N19"/>
     <mergeCell ref="C2:D2"/>
+    <mergeCell ref="I10:N10"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="A25:J25"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="H10:M10"/>
     <mergeCell ref="G1:H1"/>
-    <mergeCell ref="H4:M4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>